<commit_message>
nueva asignacion y canridad lhd
</commit_message>
<xml_diff>
--- a/data/Escenarios_DET/Swap_costo_fijo/elmo_data.xlsx
+++ b/data/Escenarios_DET/Swap_costo_fijo/elmo_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Agustin\Desktop\Elmo_infrastructure_NP\data\Escenarios_DET\Swap_costo_fijo\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TECNO-MASTER\Desktop\Elmo_infrastructure_sizing_NP-\data\Escenarios_DET\Swap_costo_fijo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0B6C9B1-2F6A-47B0-BF6B-1D0039E73B03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97A317CE-B640-43A4-91ED-AE4F0A4FDED3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LHD" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="794" uniqueCount="309">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="784" uniqueCount="307">
   <si>
     <t>id</t>
   </si>
@@ -949,12 +949,6 @@
   </si>
   <si>
     <t>LH518B_7</t>
-  </si>
-  <si>
-    <t>LH518B_8</t>
-  </si>
-  <si>
-    <t>LH518B_9</t>
   </si>
   <si>
     <t>battery_cost</t>
@@ -1813,39 +1807,39 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:AD11"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:AD9"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.44140625" style="20" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="31.33203125" style="20" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.33203125" style="20" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.5546875" style="20" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.44140625" style="20" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="6.77734375" style="62" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.5546875" style="20" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.6640625" style="21" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="13.109375" style="20" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.42578125" style="20" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="31.28515625" style="20" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.28515625" style="20" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.5703125" style="20" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.42578125" style="20" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="6.7109375" style="62" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.5703125" style="20" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.7109375" style="21" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.140625" style="20" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="15" style="20" customWidth="1"/>
-    <col min="16" max="16" width="16.88671875" style="20" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="13.77734375" style="21" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="16.85546875" style="20" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.7109375" style="21" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="18" style="21" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="20.88671875" style="21" bestFit="1" customWidth="1"/>
-    <col min="20" max="23" width="20.88671875" style="21" customWidth="1"/>
-    <col min="24" max="24" width="18.44140625" style="21" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="20.109375" style="21" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="15.21875" style="21" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="8.21875" style="21" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="16.5546875" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="19.109375" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="20.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="20" max="23" width="20.85546875" style="21" customWidth="1"/>
+    <col min="24" max="24" width="18.42578125" style="21" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="20.140625" style="21" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="15.28515625" style="21" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="8.28515625" style="21" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="10.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
@@ -1937,7 +1931,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="2" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="27" t="s">
         <v>3</v>
       </c>
@@ -2029,7 +2023,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="3" spans="1:30" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:30" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="28">
         <v>1</v>
       </c>
@@ -2040,7 +2034,7 @@
         <v>72</v>
       </c>
       <c r="D3" s="26" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="E3" s="18" t="s">
         <v>48</v>
@@ -2121,7 +2115,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="28">
         <v>2</v>
       </c>
@@ -2132,7 +2126,7 @@
         <v>72</v>
       </c>
       <c r="D4" s="26" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="E4" s="18" t="s">
         <v>48</v>
@@ -2213,7 +2207,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="28">
         <v>3</v>
       </c>
@@ -2224,7 +2218,7 @@
         <v>72</v>
       </c>
       <c r="D5" s="26" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="E5" s="18" t="s">
         <v>48</v>
@@ -2305,7 +2299,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="28">
         <v>4</v>
       </c>
@@ -2316,7 +2310,7 @@
         <v>72</v>
       </c>
       <c r="D6" s="26" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="E6" s="18" t="s">
         <v>48</v>
@@ -2397,7 +2391,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="28">
         <v>5</v>
       </c>
@@ -2408,7 +2402,7 @@
         <v>72</v>
       </c>
       <c r="D7" s="26" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="E7" s="18" t="s">
         <v>48</v>
@@ -2489,7 +2483,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="28">
         <v>6</v>
       </c>
@@ -2500,7 +2494,7 @@
         <v>72</v>
       </c>
       <c r="D8" s="26" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="E8" s="18" t="s">
         <v>48</v>
@@ -2581,7 +2575,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="28">
         <v>7</v>
       </c>
@@ -2592,7 +2586,7 @@
         <v>72</v>
       </c>
       <c r="D9" s="26" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="E9" s="18" t="s">
         <v>48</v>
@@ -2670,190 +2664,6 @@
         <v>0.95</v>
       </c>
       <c r="AD9" s="65">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A10" s="28">
-        <v>8</v>
-      </c>
-      <c r="B10" s="33" t="s">
-        <v>304</v>
-      </c>
-      <c r="C10" s="31" t="s">
-        <v>72</v>
-      </c>
-      <c r="D10" s="26" t="s">
-        <v>307</v>
-      </c>
-      <c r="E10" s="18" t="s">
-        <v>48</v>
-      </c>
-      <c r="F10" s="18" t="s">
-        <v>73</v>
-      </c>
-      <c r="G10" s="6">
-        <v>18</v>
-      </c>
-      <c r="H10" s="63">
-        <v>0.84</v>
-      </c>
-      <c r="I10" s="64">
-        <v>20</v>
-      </c>
-      <c r="J10" s="64">
-        <v>20</v>
-      </c>
-      <c r="K10" s="61">
-        <v>54.8</v>
-      </c>
-      <c r="L10" s="6">
-        <v>540</v>
-      </c>
-      <c r="M10" s="19">
-        <v>8.73</v>
-      </c>
-      <c r="N10" s="58">
-        <v>-1</v>
-      </c>
-      <c r="O10" s="58">
-        <v>-1</v>
-      </c>
-      <c r="P10" s="58">
-        <v>-1</v>
-      </c>
-      <c r="Q10" s="58">
-        <v>-1</v>
-      </c>
-      <c r="R10" s="32">
-        <v>0.95</v>
-      </c>
-      <c r="S10" s="23">
-        <v>0.92</v>
-      </c>
-      <c r="T10" s="25">
-        <v>15</v>
-      </c>
-      <c r="U10" s="66">
-        <v>0.47</v>
-      </c>
-      <c r="V10" s="31">
-        <v>160</v>
-      </c>
-      <c r="W10" s="65">
-        <v>4</v>
-      </c>
-      <c r="X10" s="57">
-        <v>320</v>
-      </c>
-      <c r="Y10" s="67">
-        <v>4</v>
-      </c>
-      <c r="Z10" s="57">
-        <v>482</v>
-      </c>
-      <c r="AA10" s="57">
-        <v>0.2</v>
-      </c>
-      <c r="AB10" s="65">
-        <v>0.95</v>
-      </c>
-      <c r="AC10" s="65">
-        <v>0.95</v>
-      </c>
-      <c r="AD10" s="65">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="11" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A11" s="28">
-        <v>9</v>
-      </c>
-      <c r="B11" s="33" t="s">
-        <v>305</v>
-      </c>
-      <c r="C11" s="31" t="s">
-        <v>72</v>
-      </c>
-      <c r="D11" s="26" t="s">
-        <v>307</v>
-      </c>
-      <c r="E11" s="18" t="s">
-        <v>48</v>
-      </c>
-      <c r="F11" s="18" t="s">
-        <v>73</v>
-      </c>
-      <c r="G11" s="6">
-        <v>18</v>
-      </c>
-      <c r="H11" s="63">
-        <v>0.84</v>
-      </c>
-      <c r="I11" s="64">
-        <v>20</v>
-      </c>
-      <c r="J11" s="64">
-        <v>20</v>
-      </c>
-      <c r="K11" s="61">
-        <v>54.8</v>
-      </c>
-      <c r="L11" s="6">
-        <v>540</v>
-      </c>
-      <c r="M11" s="19">
-        <v>8.73</v>
-      </c>
-      <c r="N11" s="58">
-        <v>-1</v>
-      </c>
-      <c r="O11" s="58">
-        <v>-1</v>
-      </c>
-      <c r="P11" s="58">
-        <v>-1</v>
-      </c>
-      <c r="Q11" s="58">
-        <v>-1</v>
-      </c>
-      <c r="R11" s="32">
-        <v>0.95</v>
-      </c>
-      <c r="S11" s="23">
-        <v>0.92</v>
-      </c>
-      <c r="T11" s="25">
-        <v>15</v>
-      </c>
-      <c r="U11" s="66">
-        <v>0.47</v>
-      </c>
-      <c r="V11" s="31">
-        <v>160</v>
-      </c>
-      <c r="W11" s="65">
-        <v>4</v>
-      </c>
-      <c r="X11" s="57">
-        <v>320</v>
-      </c>
-      <c r="Y11" s="67">
-        <v>4</v>
-      </c>
-      <c r="Z11" s="57">
-        <v>482</v>
-      </c>
-      <c r="AA11" s="57">
-        <v>0.2</v>
-      </c>
-      <c r="AB11" s="65">
-        <v>0.95</v>
-      </c>
-      <c r="AC11" s="65">
-        <v>0.95</v>
-      </c>
-      <c r="AD11" s="65">
         <v>8</v>
       </c>
     </row>
@@ -2867,15 +2677,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CC93900-5A86-4519-AB89-460E8AC441EE}">
   <dimension ref="A1:H3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="17.88671875" customWidth="1"/>
-    <col min="3" max="3" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.85546875" customWidth="1"/>
+    <col min="3" max="3" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
@@ -2895,13 +2705,13 @@
         <v>61</v>
       </c>
       <c r="G1" s="9" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="H1" s="9" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="27" t="s">
         <v>3</v>
       </c>
@@ -2927,7 +2737,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="31">
         <v>1</v>
       </c>
@@ -2963,14 +2773,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA5C58D2-31A1-4CA6-99E5-3102447D41CF}">
   <dimension ref="A1:H3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="13.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
@@ -2990,13 +2800,13 @@
         <v>69</v>
       </c>
       <c r="G1" s="9" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="H1" s="9" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="27" t="s">
         <v>3</v>
       </c>
@@ -3022,7 +2832,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="31">
         <v>1</v>
       </c>
@@ -3059,17 +2869,17 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:H236"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" style="7" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.5546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.44140625" style="8" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="29.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.5546875" style="7" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" style="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.5703125" style="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.42578125" style="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="29.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.5703125" style="7" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="40" t="s">
         <v>0</v>
       </c>
@@ -3095,7 +2905,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="45" t="s">
         <v>3</v>
       </c>
@@ -3121,7 +2931,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="52">
         <v>1</v>
       </c>
@@ -3147,7 +2957,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="52">
         <v>2</v>
       </c>
@@ -3173,7 +2983,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="52">
         <v>3</v>
       </c>
@@ -3199,7 +3009,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="52">
         <v>4</v>
       </c>
@@ -3225,7 +3035,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="52">
         <v>5</v>
       </c>
@@ -3251,7 +3061,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="52">
         <v>6</v>
       </c>
@@ -3277,7 +3087,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="52">
         <v>7</v>
       </c>
@@ -3303,7 +3113,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="52">
         <v>8</v>
       </c>
@@ -3329,7 +3139,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="52">
         <v>9</v>
       </c>
@@ -3355,7 +3165,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="52">
         <v>10</v>
       </c>
@@ -3381,7 +3191,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="52">
         <v>11</v>
       </c>
@@ -3407,7 +3217,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="52">
         <v>12</v>
       </c>
@@ -3433,7 +3243,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="52">
         <v>13</v>
       </c>
@@ -3459,7 +3269,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="52">
         <v>14</v>
       </c>
@@ -3485,7 +3295,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="52">
         <v>15</v>
       </c>
@@ -3511,7 +3321,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="52">
         <v>16</v>
       </c>
@@ -3537,7 +3347,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="52">
         <v>17</v>
       </c>
@@ -3563,7 +3373,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="52">
         <v>18</v>
       </c>
@@ -3589,7 +3399,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="52">
         <v>19</v>
       </c>
@@ -3615,7 +3425,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="52">
         <v>20</v>
       </c>
@@ -3641,7 +3451,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="52">
         <v>21</v>
       </c>
@@ -3667,7 +3477,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="52">
         <v>22</v>
       </c>
@@ -3693,7 +3503,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="52">
         <v>23</v>
       </c>
@@ -3719,7 +3529,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="52">
         <v>24</v>
       </c>
@@ -3745,7 +3555,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="52">
         <v>25</v>
       </c>
@@ -3771,7 +3581,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="52">
         <v>26</v>
       </c>
@@ -3797,7 +3607,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="52">
         <v>27</v>
       </c>
@@ -3823,7 +3633,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="52">
         <v>28</v>
       </c>
@@ -3849,7 +3659,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="52">
         <v>29</v>
       </c>
@@ -3875,7 +3685,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="52">
         <v>30</v>
       </c>
@@ -3901,7 +3711,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="52">
         <v>31</v>
       </c>
@@ -3927,7 +3737,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="52">
         <v>32</v>
       </c>
@@ -3953,7 +3763,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="52">
         <v>33</v>
       </c>
@@ -3979,7 +3789,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="52">
         <v>34</v>
       </c>
@@ -4005,7 +3815,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="52">
         <v>35</v>
       </c>
@@ -4031,7 +3841,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="52">
         <v>36</v>
       </c>
@@ -4057,7 +3867,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="52">
         <v>37</v>
       </c>
@@ -4083,7 +3893,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" s="52">
         <v>38</v>
       </c>
@@ -4109,7 +3919,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" s="52">
         <v>39</v>
       </c>
@@ -4135,7 +3945,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" s="52">
         <v>40</v>
       </c>
@@ -4161,7 +3971,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" s="52">
         <v>41</v>
       </c>
@@ -4187,7 +3997,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="52">
         <v>42</v>
       </c>
@@ -4213,7 +4023,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" s="52">
         <v>43</v>
       </c>
@@ -4239,7 +4049,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" s="52">
         <v>44</v>
       </c>
@@ -4265,7 +4075,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" s="52">
         <v>45</v>
       </c>
@@ -4291,7 +4101,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" s="52">
         <v>46</v>
       </c>
@@ -4317,7 +4127,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" s="52">
         <v>47</v>
       </c>
@@ -4343,7 +4153,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" s="52">
         <v>48</v>
       </c>
@@ -4369,7 +4179,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" s="52">
         <v>49</v>
       </c>
@@ -4395,7 +4205,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" s="52">
         <v>50</v>
       </c>
@@ -4421,7 +4231,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" s="52">
         <v>51</v>
       </c>
@@ -4447,7 +4257,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" s="52">
         <v>52</v>
       </c>
@@ -4473,7 +4283,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" s="52">
         <v>53</v>
       </c>
@@ -4499,7 +4309,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" s="52">
         <v>54</v>
       </c>
@@ -4525,7 +4335,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" s="52">
         <v>55</v>
       </c>
@@ -4551,7 +4361,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" s="52">
         <v>56</v>
       </c>
@@ -4577,7 +4387,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" s="52">
         <v>57</v>
       </c>
@@ -4603,7 +4413,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" s="52">
         <v>58</v>
       </c>
@@ -4629,7 +4439,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" s="52">
         <v>59</v>
       </c>
@@ -4655,7 +4465,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" s="52">
         <v>60</v>
       </c>
@@ -4681,7 +4491,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" s="52">
         <v>61</v>
       </c>
@@ -4707,7 +4517,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" s="52">
         <v>62</v>
       </c>
@@ -4733,7 +4543,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" s="52">
         <v>63</v>
       </c>
@@ -4759,7 +4569,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66" s="52">
         <v>64</v>
       </c>
@@ -4785,7 +4595,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" s="52">
         <v>65</v>
       </c>
@@ -4811,7 +4621,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68" s="52">
         <v>66</v>
       </c>
@@ -4837,7 +4647,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69" s="52">
         <v>67</v>
       </c>
@@ -4863,7 +4673,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70" s="52">
         <v>68</v>
       </c>
@@ -4889,7 +4699,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71" s="52">
         <v>69</v>
       </c>
@@ -4915,7 +4725,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A72" s="52">
         <v>70</v>
       </c>
@@ -4941,7 +4751,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A73" s="52">
         <v>71</v>
       </c>
@@ -4967,7 +4777,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A74" s="52">
         <v>72</v>
       </c>
@@ -4993,7 +4803,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A75" s="52">
         <v>73</v>
       </c>
@@ -5019,7 +4829,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A76" s="52">
         <v>74</v>
       </c>
@@ -5045,7 +4855,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A77" s="52">
         <v>75</v>
       </c>
@@ -5071,7 +4881,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A78" s="52">
         <v>76</v>
       </c>
@@ -5097,7 +4907,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A79" s="52">
         <v>77</v>
       </c>
@@ -5123,7 +4933,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A80" s="52">
         <v>78</v>
       </c>
@@ -5149,7 +4959,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A81" s="52">
         <v>79</v>
       </c>
@@ -5175,7 +4985,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A82" s="52">
         <v>80</v>
       </c>
@@ -5201,7 +5011,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A83" s="52">
         <v>81</v>
       </c>
@@ -5227,7 +5037,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A84" s="52">
         <v>82</v>
       </c>
@@ -5253,7 +5063,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A85" s="52">
         <v>83</v>
       </c>
@@ -5279,7 +5089,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A86" s="52">
         <v>84</v>
       </c>
@@ -5305,7 +5115,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A87" s="52">
         <v>85</v>
       </c>
@@ -5331,7 +5141,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A88" s="52">
         <v>86</v>
       </c>
@@ -5357,7 +5167,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A89" s="52">
         <v>87</v>
       </c>
@@ -5383,7 +5193,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A90" s="52">
         <v>88</v>
       </c>
@@ -5409,7 +5219,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A91" s="52">
         <v>89</v>
       </c>
@@ -5435,7 +5245,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A92" s="52">
         <v>90</v>
       </c>
@@ -5461,7 +5271,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A93" s="52">
         <v>91</v>
       </c>
@@ -5487,7 +5297,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A94" s="52">
         <v>92</v>
       </c>
@@ -5513,7 +5323,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A95" s="52">
         <v>93</v>
       </c>
@@ -5539,7 +5349,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A96" s="52">
         <v>94</v>
       </c>
@@ -5565,7 +5375,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A97" s="52">
         <v>95</v>
       </c>
@@ -5591,7 +5401,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A98" s="52">
         <v>96</v>
       </c>
@@ -5617,7 +5427,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A99" s="52">
         <v>97</v>
       </c>
@@ -5643,7 +5453,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A100" s="52">
         <v>98</v>
       </c>
@@ -5669,7 +5479,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A101" s="52">
         <v>99</v>
       </c>
@@ -5695,7 +5505,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A102" s="52">
         <v>100</v>
       </c>
@@ -5721,7 +5531,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A103" s="52">
         <v>101</v>
       </c>
@@ -5747,7 +5557,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A104" s="52">
         <v>102</v>
       </c>
@@ -5773,7 +5583,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A105" s="52">
         <v>103</v>
       </c>
@@ -5799,7 +5609,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A106" s="52">
         <v>104</v>
       </c>
@@ -5825,7 +5635,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A107" s="52">
         <v>105</v>
       </c>
@@ -5851,7 +5661,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A108" s="52">
         <v>106</v>
       </c>
@@ -5877,7 +5687,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A109" s="52">
         <v>107</v>
       </c>
@@ -5903,7 +5713,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A110" s="52">
         <v>108</v>
       </c>
@@ -5929,7 +5739,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A111" s="52">
         <v>109</v>
       </c>
@@ -5955,7 +5765,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A112" s="52">
         <v>110</v>
       </c>
@@ -5981,7 +5791,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A113" s="52">
         <v>111</v>
       </c>
@@ -6007,7 +5817,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A114" s="52">
         <v>112</v>
       </c>
@@ -6033,7 +5843,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A115" s="52">
         <v>113</v>
       </c>
@@ -6059,7 +5869,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A116" s="52">
         <v>114</v>
       </c>
@@ -6085,7 +5895,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A117" s="52">
         <v>115</v>
       </c>
@@ -6111,7 +5921,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A118" s="52">
         <v>116</v>
       </c>
@@ -6137,7 +5947,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A119" s="52">
         <v>117</v>
       </c>
@@ -6163,7 +5973,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A120" s="52">
         <v>118</v>
       </c>
@@ -6189,7 +5999,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A121" s="52">
         <v>119</v>
       </c>
@@ -6215,7 +6025,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A122" s="52">
         <v>120</v>
       </c>
@@ -6241,7 +6051,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A123" s="52">
         <v>121</v>
       </c>
@@ -6267,7 +6077,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A124" s="52">
         <v>122</v>
       </c>
@@ -6293,7 +6103,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A125" s="52">
         <v>123</v>
       </c>
@@ -6319,7 +6129,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A126" s="52">
         <v>124</v>
       </c>
@@ -6345,7 +6155,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A127" s="52">
         <v>125</v>
       </c>
@@ -6371,7 +6181,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A128" s="52">
         <v>126</v>
       </c>
@@ -6397,7 +6207,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A129" s="52">
         <v>127</v>
       </c>
@@ -6423,7 +6233,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A130" s="52">
         <v>128</v>
       </c>
@@ -6449,7 +6259,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A131" s="52">
         <v>129</v>
       </c>
@@ -6475,7 +6285,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A132" s="52">
         <v>130</v>
       </c>
@@ -6501,7 +6311,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A133" s="52">
         <v>131</v>
       </c>
@@ -6527,7 +6337,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A134" s="52">
         <v>132</v>
       </c>
@@ -6553,7 +6363,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="135" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A135" s="52">
         <v>133</v>
       </c>
@@ -6579,7 +6389,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A136" s="52">
         <v>134</v>
       </c>
@@ -6605,7 +6415,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A137" s="52">
         <v>135</v>
       </c>
@@ -6631,7 +6441,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A138" s="52">
         <v>136</v>
       </c>
@@ -6657,7 +6467,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A139" s="52">
         <v>137</v>
       </c>
@@ -6683,7 +6493,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A140" s="52">
         <v>138</v>
       </c>
@@ -6709,7 +6519,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A141" s="52">
         <v>139</v>
       </c>
@@ -6735,7 +6545,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A142" s="52">
         <v>140</v>
       </c>
@@ -6761,7 +6571,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A143" s="52">
         <v>141</v>
       </c>
@@ -6787,7 +6597,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A144" s="52">
         <v>142</v>
       </c>
@@ -6813,7 +6623,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="145" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A145" s="52">
         <v>143</v>
       </c>
@@ -6839,7 +6649,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A146" s="52">
         <v>144</v>
       </c>
@@ -6865,7 +6675,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A147" s="52">
         <v>145</v>
       </c>
@@ -6891,7 +6701,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="148" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A148" s="52">
         <v>146</v>
       </c>
@@ -6917,7 +6727,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="149" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A149" s="52">
         <v>147</v>
       </c>
@@ -6943,7 +6753,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="150" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A150" s="52">
         <v>148</v>
       </c>
@@ -6969,7 +6779,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="151" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A151" s="52">
         <v>149</v>
       </c>
@@ -6995,7 +6805,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="152" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A152" s="52">
         <v>150</v>
       </c>
@@ -7021,7 +6831,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="153" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A153" s="52">
         <v>151</v>
       </c>
@@ -7047,7 +6857,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A154" s="52">
         <v>152</v>
       </c>
@@ -7073,7 +6883,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A155" s="52">
         <v>153</v>
       </c>
@@ -7099,7 +6909,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A156" s="52">
         <v>154</v>
       </c>
@@ -7125,7 +6935,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A157" s="52">
         <v>155</v>
       </c>
@@ -7151,7 +6961,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A158" s="52">
         <v>156</v>
       </c>
@@ -7177,7 +6987,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="159" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A159" s="52">
         <v>157</v>
       </c>
@@ -7203,7 +7013,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="160" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A160" s="52">
         <v>158</v>
       </c>
@@ -7229,7 +7039,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A161" s="52">
         <v>159</v>
       </c>
@@ -7255,7 +7065,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A162" s="52">
         <v>160</v>
       </c>
@@ -7281,7 +7091,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="163" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A163" s="52">
         <v>161</v>
       </c>
@@ -7307,7 +7117,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="164" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A164" s="52">
         <v>162</v>
       </c>
@@ -7333,7 +7143,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="165" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A165" s="52">
         <v>163</v>
       </c>
@@ -7359,7 +7169,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="166" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A166" s="52">
         <v>164</v>
       </c>
@@ -7385,7 +7195,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="167" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A167" s="52">
         <v>165</v>
       </c>
@@ -7411,7 +7221,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="168" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A168" s="52">
         <v>166</v>
       </c>
@@ -7437,7 +7247,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A169" s="52">
         <v>167</v>
       </c>
@@ -7463,7 +7273,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="170" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A170" s="52">
         <v>168</v>
       </c>
@@ -7489,7 +7299,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A171" s="52">
         <v>169</v>
       </c>
@@ -7515,7 +7325,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A172" s="52">
         <v>170</v>
       </c>
@@ -7541,7 +7351,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="173" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A173" s="52">
         <v>171</v>
       </c>
@@ -7567,7 +7377,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="174" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A174" s="52">
         <v>172</v>
       </c>
@@ -7593,7 +7403,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A175" s="52">
         <v>173</v>
       </c>
@@ -7619,7 +7429,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="176" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A176" s="52">
         <v>174</v>
       </c>
@@ -7645,7 +7455,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A177" s="52">
         <v>175</v>
       </c>
@@ -7671,7 +7481,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A178" s="52">
         <v>176</v>
       </c>
@@ -7697,7 +7507,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="179" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A179" s="52">
         <v>177</v>
       </c>
@@ -7723,7 +7533,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A180" s="52">
         <v>178</v>
       </c>
@@ -7749,7 +7559,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A181" s="52">
         <v>179</v>
       </c>
@@ -7775,7 +7585,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="182" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A182" s="52">
         <v>180</v>
       </c>
@@ -7801,7 +7611,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="183" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A183" s="52">
         <v>181</v>
       </c>
@@ -7827,7 +7637,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="184" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A184" s="52">
         <v>182</v>
       </c>
@@ -7853,7 +7663,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="185" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A185" s="52">
         <v>183</v>
       </c>
@@ -7879,7 +7689,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="186" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A186" s="52">
         <v>184</v>
       </c>
@@ -7905,7 +7715,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="187" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A187" s="52">
         <v>185</v>
       </c>
@@ -7931,7 +7741,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="188" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A188" s="52">
         <v>186</v>
       </c>
@@ -7957,7 +7767,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="189" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A189" s="52">
         <v>187</v>
       </c>
@@ -7983,7 +7793,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="190" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A190" s="52">
         <v>188</v>
       </c>
@@ -8009,7 +7819,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="191" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A191" s="52">
         <v>189</v>
       </c>
@@ -8035,7 +7845,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="192" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A192" s="52">
         <v>190</v>
       </c>
@@ -8061,7 +7871,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="193" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A193" s="52">
         <v>191</v>
       </c>
@@ -8087,7 +7897,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="194" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A194" s="52">
         <v>192</v>
       </c>
@@ -8113,7 +7923,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="195" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A195" s="52">
         <v>193</v>
       </c>
@@ -8139,7 +7949,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="196" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A196" s="52">
         <v>194</v>
       </c>
@@ -8165,7 +7975,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="197" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A197" s="52">
         <v>195</v>
       </c>
@@ -8191,7 +8001,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="198" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A198" s="52">
         <v>196</v>
       </c>
@@ -8217,7 +8027,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="199" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A199" s="52">
         <v>197</v>
       </c>
@@ -8243,7 +8053,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="200" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A200" s="52">
         <v>198</v>
       </c>
@@ -8269,7 +8079,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="201" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A201" s="52">
         <v>199</v>
       </c>
@@ -8295,7 +8105,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="202" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A202" s="52">
         <v>200</v>
       </c>
@@ -8321,7 +8131,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="203" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A203" s="52">
         <v>201</v>
       </c>
@@ -8347,7 +8157,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="204" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A204" s="52">
         <v>202</v>
       </c>
@@ -8373,7 +8183,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="205" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A205" s="52">
         <v>203</v>
       </c>
@@ -8399,7 +8209,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="206" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A206" s="52">
         <v>204</v>
       </c>
@@ -8425,7 +8235,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="207" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A207" s="52">
         <v>205</v>
       </c>
@@ -8451,7 +8261,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="208" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A208" s="52">
         <v>206</v>
       </c>
@@ -8477,7 +8287,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="209" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A209" s="52">
         <v>207</v>
       </c>
@@ -8503,7 +8313,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="210" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A210" s="52">
         <v>208</v>
       </c>
@@ -8529,7 +8339,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="211" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A211" s="52">
         <v>209</v>
       </c>
@@ -8555,7 +8365,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="212" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A212" s="52">
         <v>210</v>
       </c>
@@ -8581,90 +8391,90 @@
         <v>0</v>
       </c>
     </row>
-    <row r="213" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A213"/>
       <c r="C213"/>
       <c r="D213"/>
       <c r="G213"/>
     </row>
-    <row r="214" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A214"/>
       <c r="C214"/>
       <c r="D214"/>
       <c r="G214"/>
     </row>
-    <row r="215" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A215"/>
       <c r="C215"/>
       <c r="D215"/>
       <c r="G215"/>
     </row>
-    <row r="216" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A216"/>
       <c r="C216"/>
       <c r="D216"/>
       <c r="G216"/>
     </row>
-    <row r="217" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A217"/>
       <c r="C217"/>
       <c r="D217"/>
       <c r="G217"/>
     </row>
-    <row r="218" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A218"/>
       <c r="C218"/>
       <c r="D218"/>
       <c r="G218"/>
     </row>
-    <row r="219" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A219"/>
       <c r="C219"/>
       <c r="D219"/>
       <c r="G219"/>
     </row>
-    <row r="220" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A220"/>
       <c r="C220"/>
       <c r="D220"/>
       <c r="G220"/>
     </row>
-    <row r="221" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A221"/>
       <c r="C221"/>
       <c r="D221"/>
       <c r="G221"/>
     </row>
-    <row r="222" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A222"/>
       <c r="C222"/>
       <c r="D222"/>
       <c r="G222"/>
     </row>
-    <row r="223" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A223"/>
       <c r="C223"/>
       <c r="D223"/>
       <c r="G223"/>
     </row>
-    <row r="224" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A224"/>
       <c r="C224"/>
       <c r="D224"/>
       <c r="G224"/>
     </row>
-    <row r="225" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="226" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="227" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="228" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="229" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="230" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="231" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="232" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="233" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="234" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="235" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="236" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="225" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="226" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="227" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="228" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="229" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="230" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="231" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="232" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="233" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="234" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="235" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="236" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8677,14 +8487,14 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -8695,7 +8505,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -8706,7 +8516,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>0</v>
       </c>

</xml_diff>